<commit_message>
Exercise Feishu write flow and ignore local state
</commit_message>
<xml_diff>
--- a/skills/family-finance/assets/family-finance-template.xlsx
+++ b/skills/family-finance/assets/family-finance-template.xlsx
@@ -331,6 +331,27 @@
           <t>1月</t>
         </is>
       </c>
+      <c r="Q3">
+        <f>B3+C3+D3+E3-H3-I3-J3</f>
+      </c>
+      <c r="R3">
+        <f>R2+Q3</f>
+      </c>
+      <c r="S3">
+        <f>Q3-M3-N3</f>
+      </c>
+      <c r="T3">
+        <f>T2+S3</f>
+      </c>
+      <c r="W3">
+        <f>V3*W2</f>
+      </c>
+      <c r="AB3">
+        <f>Q3+W3+X3-Y3</f>
+      </c>
+      <c r="AC3">
+        <f>AC2+AB3</f>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -338,6 +359,27 @@
           <t>2月</t>
         </is>
       </c>
+      <c r="Q4">
+        <f>B4+C4+D4+E4-H4-I4-J4</f>
+      </c>
+      <c r="R4">
+        <f>R3+Q4</f>
+      </c>
+      <c r="S4">
+        <f>Q4-M4-N4</f>
+      </c>
+      <c r="T4">
+        <f>T3+S4</f>
+      </c>
+      <c r="W4">
+        <f>V4*W2</f>
+      </c>
+      <c r="AB4">
+        <f>Q4+W4+X4-Y4</f>
+      </c>
+      <c r="AC4">
+        <f>AC3+AB4</f>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -345,6 +387,27 @@
           <t>3月</t>
         </is>
       </c>
+      <c r="Q5">
+        <f>B5+C5+D5+E5-H5-I5-J5</f>
+      </c>
+      <c r="R5">
+        <f>R4+Q5</f>
+      </c>
+      <c r="S5">
+        <f>Q5-M5-N5</f>
+      </c>
+      <c r="T5">
+        <f>T4+S5</f>
+      </c>
+      <c r="W5">
+        <f>V5*W2</f>
+      </c>
+      <c r="AB5">
+        <f>Q5+W5+X5-Y5</f>
+      </c>
+      <c r="AC5">
+        <f>AC4+AB5</f>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -352,6 +415,27 @@
           <t>4月</t>
         </is>
       </c>
+      <c r="Q6">
+        <f>B6+C6+D6+E6-H6-I6-J6</f>
+      </c>
+      <c r="R6">
+        <f>R5+Q6</f>
+      </c>
+      <c r="S6">
+        <f>Q6-M6-N6</f>
+      </c>
+      <c r="T6">
+        <f>T5+S6</f>
+      </c>
+      <c r="W6">
+        <f>V6*W2</f>
+      </c>
+      <c r="AB6">
+        <f>Q6+W6+X6-Y6</f>
+      </c>
+      <c r="AC6">
+        <f>AC5+AB6</f>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -359,6 +443,27 @@
           <t>5月</t>
         </is>
       </c>
+      <c r="Q7">
+        <f>B7+C7+D7+E7-H7-I7-J7</f>
+      </c>
+      <c r="R7">
+        <f>R6+Q7</f>
+      </c>
+      <c r="S7">
+        <f>Q7-M7-N7</f>
+      </c>
+      <c r="T7">
+        <f>T6+S7</f>
+      </c>
+      <c r="W7">
+        <f>V7*W2</f>
+      </c>
+      <c r="AB7">
+        <f>Q7+W7+X7-Y7</f>
+      </c>
+      <c r="AC7">
+        <f>AC6+AB7</f>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -366,6 +471,27 @@
           <t>6月</t>
         </is>
       </c>
+      <c r="Q8">
+        <f>B8+C8+D8+E8-H8-I8-J8</f>
+      </c>
+      <c r="R8">
+        <f>R7+Q8</f>
+      </c>
+      <c r="S8">
+        <f>Q8-M8-N8</f>
+      </c>
+      <c r="T8">
+        <f>T7+S8</f>
+      </c>
+      <c r="W8">
+        <f>V8*W2</f>
+      </c>
+      <c r="AB8">
+        <f>Q8+W8+X8-Y8</f>
+      </c>
+      <c r="AC8">
+        <f>AC7+AB8</f>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -373,6 +499,27 @@
           <t>7月</t>
         </is>
       </c>
+      <c r="Q9">
+        <f>B9+C9+D9+E9-H9-I9-J9</f>
+      </c>
+      <c r="R9">
+        <f>R8+Q9</f>
+      </c>
+      <c r="S9">
+        <f>Q9-M9-N9</f>
+      </c>
+      <c r="T9">
+        <f>T8+S9</f>
+      </c>
+      <c r="W9">
+        <f>V9*W2</f>
+      </c>
+      <c r="AB9">
+        <f>Q9+W9+X9-Y9</f>
+      </c>
+      <c r="AC9">
+        <f>AC8+AB9</f>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -380,6 +527,27 @@
           <t>8月</t>
         </is>
       </c>
+      <c r="Q10">
+        <f>B10+C10+D10+E10-H10-I10-J10</f>
+      </c>
+      <c r="R10">
+        <f>R9+Q10</f>
+      </c>
+      <c r="S10">
+        <f>Q10-M10-N10</f>
+      </c>
+      <c r="T10">
+        <f>T9+S10</f>
+      </c>
+      <c r="W10">
+        <f>V10*W2</f>
+      </c>
+      <c r="AB10">
+        <f>Q10+W10+X10-Y10</f>
+      </c>
+      <c r="AC10">
+        <f>AC9+AB10</f>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -387,6 +555,27 @@
           <t>9月</t>
         </is>
       </c>
+      <c r="Q11">
+        <f>B11+C11+D11+E11-H11-I11-J11</f>
+      </c>
+      <c r="R11">
+        <f>R10+Q11</f>
+      </c>
+      <c r="S11">
+        <f>Q11-M11-N11</f>
+      </c>
+      <c r="T11">
+        <f>T10+S11</f>
+      </c>
+      <c r="W11">
+        <f>V11*W2</f>
+      </c>
+      <c r="AB11">
+        <f>Q11+W11+X11-Y11</f>
+      </c>
+      <c r="AC11">
+        <f>AC10+AB11</f>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -394,6 +583,27 @@
           <t>10月</t>
         </is>
       </c>
+      <c r="Q12">
+        <f>B12+C12+D12+E12-H12-I12-J12</f>
+      </c>
+      <c r="R12">
+        <f>R11+Q12</f>
+      </c>
+      <c r="S12">
+        <f>Q12-M12-N12</f>
+      </c>
+      <c r="T12">
+        <f>T11+S12</f>
+      </c>
+      <c r="W12">
+        <f>V12*W2</f>
+      </c>
+      <c r="AB12">
+        <f>Q12+W12+X12-Y12</f>
+      </c>
+      <c r="AC12">
+        <f>AC11+AB12</f>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -401,12 +611,54 @@
           <t>11月</t>
         </is>
       </c>
+      <c r="Q13">
+        <f>B13+C13+D13+E13-H13-I13-J13</f>
+      </c>
+      <c r="R13">
+        <f>R12+Q13</f>
+      </c>
+      <c r="S13">
+        <f>Q13-M13-N13</f>
+      </c>
+      <c r="T13">
+        <f>T12+S13</f>
+      </c>
+      <c r="W13">
+        <f>V13*W2</f>
+      </c>
+      <c r="AB13">
+        <f>Q13+W13+X13-Y13</f>
+      </c>
+      <c r="AC13">
+        <f>AC12+AB13</f>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
           <t>12月</t>
         </is>
+      </c>
+      <c r="Q14">
+        <f>B14+C14+D14+E14-H14-I14-J14</f>
+      </c>
+      <c r="R14">
+        <f>R13+Q14</f>
+      </c>
+      <c r="S14">
+        <f>Q14-M14-N14</f>
+      </c>
+      <c r="T14">
+        <f>T13+S14</f>
+      </c>
+      <c r="W14">
+        <f>V14*W2</f>
+      </c>
+      <c r="AB14">
+        <f>Q14+W14+X14-Y14</f>
+      </c>
+      <c r="AC14">
+        <f>AC13+AB14</f>
       </c>
     </row>
     <row r="15"/>

</xml_diff>

<commit_message>
Fix family finance template formulas
</commit_message>
<xml_diff>
--- a/skills/family-finance/assets/family-finance-template.xlsx
+++ b/skills/family-finance/assets/family-finance-template.xlsx
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="Q16">
-        <f>B16-H16</f>
+        <f>SUM(Q3:Q14)</f>
       </c>
       <c r="U16" t="inlineStr">
         <is>
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="Q17">
-        <f>Q16-M17</f>
+        <f>SUM(S3:S14)</f>
       </c>
       <c r="U17" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
         </is>
       </c>
       <c r="AB17">
-        <f>Q16+V17</f>
+        <f>SUM(AB3:AB14)</f>
       </c>
     </row>
     <row r="18">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="H2">
-        <f>SUM(H3:H10)</f>
+        <f>SUM(H3:H6)</f>
       </c>
       <c r="I2">
         <v>0.4</v>
@@ -934,7 +934,7 @@
         </is>
       </c>
       <c r="H3">
-        <f>DIVIDE(G3,G18)</f>
+        <f>IFERROR(DIVIDE(G3,G13),0)</f>
       </c>
       <c r="I3">
         <v>0.05</v>
@@ -957,7 +957,7 @@
         </is>
       </c>
       <c r="H4">
-        <f>DIVIDE(G4,G18)</f>
+        <f>IFERROR(DIVIDE(G4,G13),0)</f>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -972,7 +972,7 @@
         </is>
       </c>
       <c r="H5">
-        <f>DIVIDE(G5,G18)</f>
+        <f>IFERROR(DIVIDE(G5,G13),0)</f>
       </c>
       <c r="I5">
         <v>0.15</v>
@@ -990,7 +990,7 @@
         </is>
       </c>
       <c r="H6">
-        <f>DIVIDE(G6,G18)</f>
+        <f>IFERROR(DIVIDE(G6,G13),0)</f>
       </c>
       <c r="I6">
         <v>0.2</v>
@@ -1008,7 +1008,7 @@
         </is>
       </c>
       <c r="H7">
-        <f>SUM(H12:H14)</f>
+        <f>SUM(H8:H9)</f>
       </c>
       <c r="I7">
         <v>0.4</v>
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="H8">
-        <f>DIVIDE(G12,G18)</f>
+        <f>IFERROR(DIVIDE(G8,G13),0)</f>
       </c>
       <c r="I8">
         <v>0.28</v>
@@ -1034,7 +1034,7 @@
         </is>
       </c>
       <c r="H9">
-        <f>DIVIDE(G13,G18)</f>
+        <f>IFERROR(DIVIDE(G9,G13),0)</f>
       </c>
     </row>
     <row r="10">
@@ -1044,7 +1044,7 @@
         </is>
       </c>
       <c r="H10">
-        <f>SUM(H16:H17)</f>
+        <f>SUM(H11:H12)</f>
       </c>
       <c r="I10">
         <v>0.2</v>
@@ -1057,7 +1057,7 @@
         </is>
       </c>
       <c r="H11">
-        <f>DIVIDE(G16,G18)</f>
+        <f>IFERROR(DIVIDE(G11,G13),0)</f>
       </c>
       <c r="I11">
         <v>0.2</v>
@@ -1070,7 +1070,7 @@
         </is>
       </c>
       <c r="H12">
-        <f>DIVIDE(G17,G18)</f>
+        <f>IFERROR(DIVIDE(G12,G13),0)</f>
       </c>
     </row>
     <row r="13">
@@ -1079,8 +1079,8 @@
           <t>负债总计</t>
         </is>
       </c>
-      <c r="B13">
-        <f>SUM(C2:C17)</f>
+      <c r="C13">
+        <f>SUM(C2:C12)</f>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1088,10 +1088,10 @@
         </is>
       </c>
       <c r="F13">
-        <f>SUM(F3:F17)</f>
+        <f>SUM(F3:F12)</f>
       </c>
       <c r="G13">
-        <f>SUM(G3:G17)</f>
+        <f>SUM(G3:G12)</f>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -1099,10 +1099,10 @@
         </is>
       </c>
       <c r="L13">
-        <f>SUM(L2:L17)</f>
+        <f>SUM(L2:L12)</f>
       </c>
       <c r="M13">
-        <f>SUM(M2:M17)</f>
+        <f>SUM(M2:M12)</f>
       </c>
     </row>
     <row r="14">
@@ -1112,7 +1112,7 @@
         </is>
       </c>
       <c r="L14">
-        <f>-B18+G18+M18</f>
+        <f>-C13+G13+M13</f>
       </c>
     </row>
   </sheetData>

</xml_diff>